<commit_message>
scan: seg8 2026-09-28 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq0_2026-09-24.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>73.2494009009222</v>
+        <v>73.24940089713421</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>21.23406136909598</v>
+        <v>21.23406136441943</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.293308049986691</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>2.622779574925215</v>
+        <v>2.622779575028248</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>71.93421175072548</v>
+        <v>71.93421174659102</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>22.0723772955761</v>
+        <v>22.07237727964426</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>3.901537033419154</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.686370188828316</v>
+        <v>1.686370188848911</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>59.6765729822414</v>
+        <v>59.67657298272631</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>13.51553049916299</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>15.21194791518491</v>
+        <v>15.21194791528774</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>71.58537853289238</v>
+        <v>71.58537853934436</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>40.47473349235283</v>
+        <v>40.47473351564403</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>8.311928846995031</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.1328229290529609</v>
+        <v>0.1328229290632639</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>63.8099921824337</v>
+        <v>63.80999220766923</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>14.03241904260573</v>
+        <v>14.03241909099157</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.206221100290863</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.5600901213900992</v>
+        <v>0.560090121534342</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>67.59721182123367</v>
+        <v>67.59721174607232</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>33.09853458622841</v>
+        <v>33.09853461484955</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.995690004046945</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.2105685495930419</v>
+        <v>0.210568549757885</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61.35529135631157</v>
+        <v>61.35529134140923</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>13.58202637617289</v>
+        <v>13.58202639286883</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>5.511657253808084</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.3536571110957957</v>
+        <v>0.3536571111679204</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>81.41686228141438</v>
+        <v>81.41686234123353</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>48.71896323758486</v>
+        <v>48.71896325140792</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.3241168937880656</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>9.407879168325769</v>
+        <v>9.40787916760457</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>63.75469564826621</v>
+        <v>63.75469561231942</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>19.27932415045887</v>
+        <v>19.2793242088593</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.749849862432089</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.5148445878043026</v>
+        <v>0.5148445878970308</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>830.5456478998648</v>
+        <v>830.5456478998524</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>49.2</v>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>52.76126834407864</v>
+        <v>52.76126834636691</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>11.20586423457042</v>
+        <v>11.20586424630999</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>3.242721414875198</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.3070866560613785</v>
+        <v>0.3070866560819811</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.59678976466345</v>
+        <v>58.59678976234009</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>31.57095682987072</v>
+        <v>31.5709568298707</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.3901962669513295</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.0458316931249114</v>
+        <v>0.0458316930630742</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>55.53010201255749</v>
+        <v>55.53010203568012</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>21.93328938499531</v>
+        <v>21.933289471873</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.2168997022357052</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-3.379297776365735</v>
+        <v>-3.379297777396037</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>704.9618442294221</v>
+        <v>704.9618442294222</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>1530</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>61.87309184582474</v>
+        <v>61.87309184245503</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>34.20577966680563</v>
+        <v>34.20577973231899</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.6970144872042183</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>28.05741354223423</v>
+        <v>28.05741354192509</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>53.46442235521511</v>
+        <v>53.46442239229288</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>22.34514887289112</v>
+        <v>22.34514888309716</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.28726384380385</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.3274220022649066</v>
+        <v>0.327422002244307</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51.27258094435848</v>
+        <v>51.27258097073213</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>16.54533653515736</v>
+        <v>16.54533653515735</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.609790548092301</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-0.1184136684245886</v>
+        <v>-0.118413669145831</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>59.44050907181794</v>
+        <v>59.44050911246213</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>31.16355498142732</v>
+        <v>31.16355515492781</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4701780665709106</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.3116141345462205</v>
+        <v>0.3116141344947039</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>642.0189914406776</v>
+        <v>642.0189914406777</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>139</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>64.34719363555132</v>
+        <v>64.34719364001188</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>18.76718807115402</v>
+        <v>18.76718807043834</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.338729368901232</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.971615790917891</v>
+        <v>1.971615790969407</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>66.48041227334613</v>
+        <v>66.48041229773915</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>18.78846762611366</v>
+        <v>18.78846758642689</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>3.149173955296404</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>1.08032653188134</v>
+        <v>1.080326531798915</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>59.91629659987021</v>
+        <v>59.91629660292053</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>40.68170857721296</v>
+        <v>40.68170850724233</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.4819305978692461</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-0.6139914817778536</v>
+        <v>-0.6139914814953231</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>60.29870083411132</v>
+        <v>60.29870054369046</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>24.98394623052076</v>
+        <v>24.98394644805045</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>2.362406059829026</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.2500403365859585</v>
+        <v>0.250040336967168</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>48.08966603315485</v>
+        <v>48.08966605636832</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>10.45839239748224</v>
+        <v>10.45839242274422</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.8142018610892848</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>2.133042001992995</v>
+        <v>2.133042001704514</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>53.94947898566538</v>
+        <v>53.94947898935146</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>13.55749932302824</v>
+        <v>13.55749930884872</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.9492122845521752</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>45.45331479053494</v>
+        <v>45.45331487266832</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>20.63506332631947</v>
+        <v>20.63506351987064</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.2756028258529526</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.6882024392353072</v>
+        <v>0.6882024399416053</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>54.56344157988064</v>
+        <v>54.56344158402709</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>10.99413267444481</v>
+        <v>10.99413261058669</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.518855424708676</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.3153477078177985</v>
+        <v>0.315347707807491</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>51.05015066869269</v>
+        <v>51.05015064328549</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>14.84682922681173</v>
+        <v>14.8468292270806</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.4210493135108956</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.3058138468467594</v>
+        <v>0.305813846990998</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>60.37878696534589</v>
+        <v>60.37878687716567</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>31.9947418485358</v>
+        <v>31.99474186974892</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.9532313968758288</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.0520269844945815</v>
+        <v>-0.0520269841545852</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.8572520668354652</v>
+        <v>0.8572520668457677</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>529.6376944217164</v>
+        <v>529.6376944217168</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>19.25</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>59.44043082626155</v>
+        <v>59.44043087441133</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>22.34597005640629</v>
+        <v>22.34597006240138</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.5206724268611933</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.2270408488563247</v>
+        <v>0.2270408488769301</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>50.91582475284383</v>
+        <v>50.91582480568743</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>18.10460676826046</v>
+        <v>18.10460676826045</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.7964605535242709</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.7698325274903475</v>
+        <v>0.7698325272842919</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>38.48379655806574</v>
+        <v>38.48379675166533</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26.49663409790027</v>
+        <v>26.49663408540461</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.5560296467548363</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.2317393880913805</v>
+        <v>0.2317393876792808</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>49.13971225824693</v>
+        <v>49.13971229947617</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>12.38334524110582</v>
+        <v>12.38334522544788</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.5217884528449944</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>1.555993211263157</v>
+        <v>1.55599321116014</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>55.89240613677791</v>
+        <v>55.89240615643908</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.90917218137598</v>
+        <v>31.90917240461783</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.1014843986670705</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.1018349676825809</v>
+        <v>0.1018349689189352</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>506.2219034568391</v>
+        <v>506.2219034568387</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>110.5</v>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46.85430281722648</v>
+        <v>46.85430270615146</v>
       </c>
       <c r="I34" s="2" t="n">
         <v>17.43990615206165</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.4526778718153634</v>
+        <v>0.4526778719183997</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>52.55482961933586</v>
+        <v>52.55482960313283</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>10.84778783287357</v>
+        <v>10.84778783566414</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.903921945478976</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.4393550310452483</v>
+        <v>0.4393550312204001</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>58.35674108667759</v>
+        <v>58.35674115005514</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>31.9218768729769</v>
+        <v>31.9218768695878</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.2089355531113578</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.2017804222707404</v>
+        <v>-0.2017804227858861</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>500.997570430627</v>
+        <v>500.9975704306268</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>20.45</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>57.62345487708932</v>
+        <v>57.6234546912795</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>18.29721113769536</v>
+        <v>18.29721115164431</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.6338296315688829</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.0952041035151308</v>
+        <v>0.0952041036387674</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>52.2145960680386</v>
+        <v>52.2145962451758</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>18.59694257990841</v>
+        <v>18.59694262550056</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.6853668817061258</v>
@@ -2516,7 +2516,7 @@
         <v>54.59075887482246</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>39.45608884410386</v>
+        <v>39.45608897673502</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>1.039383937338668</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.2401357160219019</v>
+        <v>0.2401357160940213</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>51.01260323796529</v>
+        <v>51.01260325679139</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>19.71298527098939</v>
+        <v>19.71298532550243</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.422985645245699</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>48.78718444626351</v>
+        <v>48.78718445367038</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>8.687098780959127</v>
+        <v>8.687098737587711</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.3914434129267762</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.264049595507362</v>
+        <v>0.2640495954867552</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>35.81790085659955</v>
+        <v>35.81790100832761</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>29.13454030690105</v>
+        <v>29.13454026646765</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.3141820252078131</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.1478936150137384</v>
+        <v>0.147893614684037</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>450.4610665738926</v>
+        <v>450.4610665738932</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>136.5</v>
@@ -2725,7 +2725,7 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>58.00829264885274</v>
+        <v>58.00829269030418</v>
       </c>
       <c r="I43" s="2" t="n">
         <v>21.86469606300656</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.5300908393068999</v>
+        <v>0.5300908392038342</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>48.44972129940726</v>
+        <v>48.44972142045864</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>10.95986967177135</v>
+        <v>10.95986967101885</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.4941303244122554</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.1681583955206962</v>
+        <v>0.168158395458887</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>27.60057457329511</v>
+        <v>27.60057458792417</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>36.30883207454902</v>
+        <v>36.30883208186607</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.7889698979822034</v>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>444.1283470648082</v>
+        <v>444.1283470648083</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>15.75</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>84.50422022791071</v>
+        <v>84.50422022572762</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>29.10211639113176</v>
+        <v>29.10211669148835</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.308481538430994</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.962996431071674</v>
+        <v>0.9629964311069878</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>436.8096555749293</v>
+        <v>436.8096555749292</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>146</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>38.14435748756608</v>
+        <v>38.14435758542266</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>31.9144813164481</v>
+        <v>31.91448136341427</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.9161167786870856</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.934316188250956</v>
+        <v>0.9343161888691612</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>17.52989326392115</v>
+        <v>17.52989328974989</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>25.97120660693966</v>
+        <v>25.9712066593548</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.523174251089526</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.92792839176199</v>
+        <v>-0.9279283909892728</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3046,7 +3046,7 @@
         <v>45.8344762770757</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>10.05367948743807</v>
+        <v>10.05367948770428</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.3889335063921308</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.1697988819073619</v>
+        <v>-0.1697988818661531</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>433.1132593159585</v>
+        <v>433.1132593159586</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>49.7</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>49.39066394941396</v>
+        <v>49.39066389075447</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>14.56543518528914</v>
+        <v>14.56543519005132</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.8553417803000599</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.0392992678491386</v>
+        <v>-0.0392992676946001</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>42.3779773361235</v>
+        <v>42.37797740029435</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>14.2988206836622</v>
+        <v>14.29882069657826</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.5547481738671958</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0233747738613289</v>
+        <v>0.023374773851028</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>39.11594063971788</v>
+        <v>39.11594069553625</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.01385830823834</v>
+        <v>22.01385831283155</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.4660050178545917</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.3324459167315483</v>
+        <v>-0.3324459166800244</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>425.064957725281</v>
+        <v>425.0649577252809</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>33.1</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>54.00722436253349</v>
+        <v>54.00722430554455</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>13.42631280819226</v>
+        <v>13.42631286137498</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5849108453482424</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0457724161039893</v>
+        <v>0.0457724161142892</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>44.2116945442697</v>
+        <v>44.21169467285982</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>15.66783781433858</v>
+        <v>15.6678378177548</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.009134458529496</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0921394500159563</v>
+        <v>0.09213944991292621</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>49.37841334316214</v>
+        <v>49.37841332368541</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>30.9561249551571</v>
+        <v>30.95612488651591</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.056874129848251</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.0153601457781634</v>
+        <v>-0.0153601457678621</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>51.51271464427377</v>
+        <v>51.51271464809114</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>15.87323203725884</v>
+        <v>15.87323203621415</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6350891145931218</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.32676968286764</v>
+        <v>46.32676966813008</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>34.87387265873591</v>
+        <v>34.87387267196713</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>3.23385898973558</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>26.65100551443807</v>
+        <v>26.65100557289973</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>39.7298797968036</v>
+        <v>39.7298797801257</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>3.649309215180266</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.1075793432954856</v>
+        <v>-0.1075793432542724</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>44.90268853590609</v>
+        <v>44.90268845807435</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>19.14537592733352</v>
+        <v>19.14537597398637</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.870816255095116</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.0686206104778504</v>
+        <v>0.06862061057398899</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>395.806233739864</v>
+        <v>395.8062337398636</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>53.3</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>53.54616959733844</v>
+        <v>53.54616935921616</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>20.46370667098736</v>
+        <v>20.46370675379365</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.3461832113339587</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.5780893469028902</v>
+        <v>0.5780893472119788</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>44.80763054786164</v>
+        <v>44.80763023937629</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>22.13862433834738</v>
+        <v>22.13862430440547</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.1275646995738436</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.0006881317697707</v>
+        <v>-0.0006881317079537</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>385.7957275390552</v>
+        <v>385.7957275390566</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>84.59999999999999</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>52.29123175580979</v>
+        <v>52.29123187603965</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>13.92391950789765</v>
+        <v>13.92391950789764</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.4376415564543019</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.5797672182628036</v>
+        <v>0.5797672178506749</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>37.8742368465935</v>
+        <v>37.87423674067127</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>26.00549270014056</v>
+        <v>26.00549275485535</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.7153699446212035</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.7004082729467176</v>
+        <v>-0.7004082722255309</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>29.44608670387028</v>
+        <v>29.44608675179266</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>17.94064225266356</v>
+        <v>17.94064223196193</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>2.743210519748104</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.0797965342746236</v>
+        <v>-0.07979653428492681</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>44.39218744026726</v>
+        <v>44.39218755379932</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>24.47278556616021</v>
+        <v>24.47278566422833</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.3123713669135161</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.1180622096157476</v>
+        <v>0.1180622097301943</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>365.5205522850395</v>
+        <v>365.5205522850393</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>372.5</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>50.21235919762609</v>
+        <v>50.21235909664376</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>14.87762758122192</v>
+        <v>14.87762766498431</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.4737584346274077</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0178239369761772</v>
+        <v>0.0178239395518524</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>362.9183820043777</v>
+        <v>362.918382004378</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>200</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>37.59374281546905</v>
+        <v>37.5937428339412</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>14.08524616133181</v>
+        <v>14.08524622068115</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.5345566382649994</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-1.382037487366118</v>
+        <v>-1.382037487489757</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.009565803573635999</v>
+        <v>0.0095658035633331</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>45.46852632295873</v>
+        <v>45.4685263260832</v>
       </c>
       <c r="I69" s="2" t="n">
         <v>19.50820935580382</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-6.479680302778668</v>
+        <v>-6.479680302953822</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>63.31744493687175</v>
+        <v>63.31744515112216</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>24.26062797254159</v>
+        <v>24.26062797343563</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.8319893985992698</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.6023967721896929</v>
+        <v>0.602396771924833</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>39.94508763918115</v>
+        <v>39.94508779821312</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>10.85102128346563</v>
+        <v>10.85102128183244</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>1.639268796293905</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.1751220949874258</v>
+        <v>-0.1751220949256044</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>39.99564330130967</v>
+        <v>39.99564296981912</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>12.69420559827619</v>
+        <v>12.69420564312602</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.2304158707798676</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0136642310999017</v>
+        <v>0.0136642316974699</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>48.51368787843401</v>
+        <v>48.51368793679789</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.41996239182416</v>
+        <v>14.41996240304545</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5661568193279873</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>324.0653797337835</v>
+        <v>324.0653797337834</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>47.05</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>48.07242044143032</v>
+        <v>48.07242049017137</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>4.145683060722592</v>
+        <v>4.145683057586741</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.2683088038008233</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.1784949683348234</v>
+        <v>-0.1784949681699747</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>49.23799440065125</v>
+        <v>49.23799436999335</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>14.05429559542204</v>
+        <v>14.05429551752357</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.445763561849045</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.1408165625014444</v>
+        <v>-0.1408165623425273</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>53.52631441600278</v>
+        <v>53.52631451143581</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>23.99762033821302</v>
+        <v>23.99762039925318</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.4103483784851667</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.007977763702887299</v>
+        <v>-0.0079777637337949</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>37.81261876128657</v>
+        <v>37.81261868001484</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>21.42950272538906</v>
+        <v>21.42950274884439</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.4644478450351711</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.358876862689568</v>
+        <v>-0.358876862792586</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>39.93312487323447</v>
+        <v>39.93312466672375</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>10.24727611709203</v>
+        <v>10.24727622473863</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.7516525806234273</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.0658733112614943</v>
+        <v>-0.0658733109083447</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>49.16335521034982</v>
+        <v>49.16335520934196</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7.246640427441988</v>
+        <v>7.24664055793403</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>3.345345107511979</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.3995026818287236</v>
+        <v>0.3995026818081206</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.15242465583187</v>
+        <v>42.15242467027045</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>24.42146598086225</v>
+        <v>24.42146607147134</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.9397689835009752</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0410481149867843</v>
+        <v>0.0410481150486006</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>51.21914756833129</v>
+        <v>51.21914761923617</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>10.43097167540313</v>
+        <v>10.43097166609611</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.3878861441404991</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>3.728766879015336</v>
+        <v>3.728766872936596</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>48.3242530629233</v>
+        <v>48.32425290956479</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>21.5821822692484</v>
+        <v>21.58218233772048</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.681370007962677</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.0222265795594587</v>
+        <v>-0.0222265795079443</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>293.4227255962332</v>
+        <v>293.4227255962333</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>20.25</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>54.23503456658418</v>
+        <v>54.23503458490082</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>12.44793140428021</v>
+        <v>12.44793143758672</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.6877823844440697</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0352277484880149</v>
+        <v>0.0352277485601328</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>292.1749118199094</v>
+        <v>292.1749118199098</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>28.05</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>42.55863155154446</v>
+        <v>42.55863151753066</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>42.72641302749053</v>
+        <v>42.72641316036842</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.3932362014188735</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.1363682499785251</v>
+        <v>-0.1363682499579219</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.3620178203756</v>
+        <v>47.36201773216294</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>15.23019305074953</v>
+        <v>15.23019304094662</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.5436892434893971</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.2053828621669871</v>
+        <v>0.2053828622081999</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>286.8794301485564</v>
+        <v>286.8794301485563</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>39.4</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>39.1919991949024</v>
+        <v>39.19199908639152</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>30.92056729872734</v>
+        <v>30.92056735080586</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4600448014237869</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.0868122733626104</v>
+        <v>-0.0868122731771603</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>283.2902910665771</v>
+        <v>283.2902910665772</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>897</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>39.97071569159002</v>
+        <v>39.97071587968107</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>18.65834525582176</v>
+        <v>18.6583454423136</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.444930927993597</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>4.895038590433515</v>
+        <v>4.895038579615424</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>275.1305447260359</v>
+        <v>275.1305447260356</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>22.1</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.40131515976681</v>
+        <v>50.40131516414796</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>9.462408573772196</v>
+        <v>9.462408584554872</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.362856786976976</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.2925903560956828</v>
+        <v>0.292590356136892</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>44.96081858521227</v>
+        <v>44.96081753811517</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>7.444581350683201</v>
+        <v>7.444581354142318</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.325644556652131</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.1218043635544516</v>
+        <v>-0.1218043634720291</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>37.20028006502795</v>
+        <v>37.20028003686538</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>17.52253043746953</v>
+        <v>17.52253043556248</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3903558381112108</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.0994180636133947</v>
+        <v>-0.09941806359279071</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>263.520905546164</v>
+        <v>263.5209055461641</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>9.19</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.0540444505513346</v>
+        <v>-0.0540444505472132</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>260.8136734565915</v>
+        <v>260.8136734565914</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>4.97</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.44134781203928</v>
+        <v>41.44134766064969</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>11.72281962953794</v>
+        <v>11.72281974578208</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.5838453257311198</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0003529155552315</v>
+        <v>0.000352915573778</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>258.5109764670898</v>
+        <v>258.5109764670899</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>32.6</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>54.62830505687006</v>
+        <v>54.62830472869088</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>21.71122315309817</v>
+        <v>21.711223276586</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.5051521165819309</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.2944629116017432</v>
+        <v>0.2944629124362764</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>255.8757996902369</v>
+        <v>255.875799690237</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>239</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>42.15212424155798</v>
+        <v>42.15212434322965</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>10.22696194278337</v>
+        <v>10.22696184385858</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.6874965859140107</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.6320824976093906</v>
+        <v>0.6320824964760692</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>248.6730044516941</v>
+        <v>248.6730044516942</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>19.5</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.77982154320085</v>
+        <v>44.77982143445032</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>8.390137058134201</v>
+        <v>8.390137098795051</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.245561382279997</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0439821996882172</v>
+        <v>0.0439821997500337</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>246.6614371408466</v>
+        <v>246.6614371408465</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>12.9</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>49.19606367004462</v>
+        <v>49.19606336536266</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>14.776671166615</v>
+        <v>14.77667112214393</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.7997761087847904</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0314301623479377</v>
+        <v>0.0314301622346051</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>236.4057042949886</v>
+        <v>236.4057042949894</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>75.3</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>37.77160707861955</v>
+        <v>37.77160691931539</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>9.398379738372276</v>
+        <v>9.398379834089996</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.5825787599634195</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.3036527543641405</v>
+        <v>-0.3036527534780893</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>42.3943240484327</v>
+        <v>42.39432402529686</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.44583043262179</v>
+        <v>19.44583043540398</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.2746056498663073</v>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>49.27768882293476</v>
+        <v>49.27768869904094</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>11.10051424083116</v>
+        <v>11.10051421895303</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4367841844436976</v>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>221.7109784126368</v>
+        <v>221.7109784126366</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>60.4</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>28.4966941024148</v>
+        <v>28.49669415520654</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>24.98660341159277</v>
+        <v>24.98660349158245</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>1.114162322787678</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.1237534031755712</v>
+        <v>-0.1237534030931438</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>44.68622252491141</v>
+        <v>44.68622278483763</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>9.332393912105202</v>
+        <v>9.332393963251448</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.2162697450883984</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.7027044999174774</v>
+        <v>0.7027044996083918</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>212.1969358151017</v>
+        <v>212.1969358151012</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>13.55</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>24.54647968221848</v>
+        <v>24.54647942493584</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>41.99963452682732</v>
+        <v>41.99963469366903</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.5310955820293388</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.07600362653059679</v>
+        <v>-0.0760036264172663</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>202.5490622151448</v>
+        <v>202.549062215144</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>5.89</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>38.14936232060218</v>
+        <v>38.14936230372392</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>6.846930116590903</v>
+        <v>6.846930116590902</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.7314112182093602</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0029180323800802</v>
+        <v>-0.002918032386262</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>198.0694103217369</v>
+        <v>198.0694103217371</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>39.35</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>46.09363191674291</v>
+        <v>46.09363210247465</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>19.94950433071456</v>
+        <v>19.94950435419418</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.3511471031230672</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.219841052890639</v>
+        <v>0.2198410525403364</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,7 +6011,7 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>49.54884800836133</v>
+        <v>49.54884807764718</v>
       </c>
       <c r="I105" s="2" t="n">
         <v>5.337048992811719</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.6725043830410813</v>
+        <v>0.6725043825877528</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>49.64938648419604</v>
+        <v>49.6493864620535</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>19.08263471436121</v>
+        <v>19.08263474226872</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.5495948264807</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0385472033606773</v>
+        <v>-0.0385472033091658</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>161.3857762199492</v>
+        <v>161.3857762199506</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>23</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>36.18675114089994</v>
+        <v>36.18675101559953</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>8.986110914268219</v>
+        <v>8.986110963551734</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.893659418827158</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.0297630656680485</v>
+        <v>-0.0297630655547189</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>157.1080846606433</v>
+        <v>157.1080846606431</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>90</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>33.45243362621748</v>
+        <v>33.45243353613918</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>18.4818099045699</v>
+        <v>18.48180991696254</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.896578083115382</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.3328505608938497</v>
+        <v>-0.3328505606053737</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>149.8091051196775</v>
+        <v>149.8091051196774</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>51</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>43.72465872717503</v>
+        <v>43.72465858264421</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>18.52092537010256</v>
+        <v>18.5209253213688</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.5276458726983252</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.1175650208643037</v>
+        <v>0.1175650213485337</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>38.27480374165346</v>
+        <v>38.27480375700789</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>12.68226075577515</v>
+        <v>12.6822608357452</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.5723249928578833</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.1690291714872818</v>
+        <v>0.1690291715078911</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>140.598632689628</v>
+        <v>140.5986326896281</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>23.85</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.99380959395561</v>
+        <v>44.99380961031101</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>15.63720281020876</v>
+        <v>15.63720279968348</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.2395428548505835</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1369212734927388</v>
+        <v>0.1369212736060691</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>45.39913031018902</v>
+        <v>45.39913048590408</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>18.10598993168044</v>
+        <v>18.10598995760498</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.8672114889065011</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.0318615843501482</v>
+        <v>-0.0318615844428749</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>41.91379305479384</v>
+        <v>41.91379303473207</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>14.48992266950823</v>
+        <v>14.48992259528953</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6894388878350682</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0357975574270632</v>
+        <v>0.0357975575094761</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>110.6111934021033</v>
+        <v>110.6111934021031</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>15</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>47.42784316902973</v>
+        <v>47.42784351015117</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>9.46774182217017</v>
+        <v>9.467741822170172</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.3103001592981505</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.0435106232693981</v>
+        <v>0.0435106232384894</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>89.01903852085734</v>
+        <v>89.01903852085742</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>139.5</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.64614061002078</v>
+        <v>39.64614018545959</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>8.293373504501654</v>
+        <v>8.293373572828507</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.8931317648877506</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0143216902165468</v>
+        <v>0.0143216914529054</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>51.17171199601122</v>
+        <v>51.17171169739495</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>17.29657450226235</v>
+        <v>17.29657476797866</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.3036550859683092</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1788009438098842</v>
+        <v>-0.1788009435729169</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg8 2026-09-29 00:36 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq0_2026-09-24.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>73.24940089713421</v>
+        <v>73.24940089052922</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>21.23406136441943</v>
+        <v>21.23406128699409</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.293308049986691</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>2.622779575028248</v>
+        <v>2.622779575050497</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>71.93421174659102</v>
+        <v>71.93421175229314</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>22.07237727964426</v>
+        <v>22.07237729799601</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>3.901537033419154</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.686370188848911</v>
+        <v>1.686370188826666</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>59.67657298272631</v>
+        <v>59.67657297627205</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>13.51553049916299</v>
+        <v>13.51553048725628</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>1.127985515119764</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>15.21194791528774</v>
+        <v>15.2119479155102</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>71.58537853934436</v>
+        <v>71.58537852544779</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>40.47473351564403</v>
+        <v>40.47473355832259</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>8.311928846995031</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.1328229290632639</v>
+        <v>0.1328229290855188</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>63.80999220766923</v>
+        <v>63.80999214080001</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>14.03241909099157</v>
+        <v>14.03241927860371</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.206221100290863</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.560090121534342</v>
+        <v>0.5600901218236456</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>67.59721174607232</v>
+        <v>67.59721168438961</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>33.09853461484955</v>
+        <v>33.09853451156518</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.995690004046945</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.210568549757885</v>
+        <v>0.2105685497690128</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61.35529134140923</v>
+        <v>61.35529133139286</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>13.58202639286883</v>
+        <v>13.58202638819264</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>5.511657253808084</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.3536571111679204</v>
+        <v>0.3536571111456604</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>81.41686234123353</v>
+        <v>81.41686224424764</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>48.71896325140792</v>
+        <v>48.71896329079097</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.3241168937880656</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>9.40787916760457</v>
+        <v>9.407879170942708</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -979,7 +979,7 @@
         <v>63.75469561231942</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>19.2793242088593</v>
+        <v>19.27932420950772</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.749849862432089</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.5148445878970308</v>
+        <v>0.5148445878747752</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>830.5456478998524</v>
+        <v>830.5456478998651</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>49.2</v>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>52.76126834636691</v>
+        <v>52.76126834326253</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>11.20586424630999</v>
+        <v>11.20586413880293</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>3.242721414875198</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.3070866560819811</v>
+        <v>0.3070866562377645</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>58.59678976234009</v>
+        <v>58.59678973606815</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>31.5709568298707</v>
+        <v>31.57095680281022</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.3901962669513295</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.0458316930630742</v>
+        <v>0.045831692974056</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>55.53010203568012</v>
+        <v>55.53010203433316</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>21.933289471873</v>
+        <v>21.93328947607357</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.2168997022357052</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-3.379297777396037</v>
+        <v>-3.379297776728404</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>61.87309184245503</v>
+        <v>61.87309184859755</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>34.20577973231899</v>
+        <v>34.20577975423276</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.6970144872042183</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>28.05741354192509</v>
+        <v>28.05741354081244</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>53.46442239229288</v>
+        <v>53.46442235585187</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>22.34514888309716</v>
+        <v>22.3451488830706</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.28726384380385</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.327422002244307</v>
+        <v>0.3274220025113684</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>51.27258097073213</v>
+        <v>51.27258093875729</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>16.54533653515735</v>
+        <v>16.54533650340321</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.609790548092301</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-0.118413669145831</v>
+        <v>-0.1184136690345777</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>59.44050911246213</v>
+        <v>59.44050909604103</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>31.16355515492781</v>
+        <v>31.16355517239214</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4701780665709106</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.3116141344947039</v>
+        <v>0.3116141345614686</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>64.34719364001188</v>
+        <v>64.34719362887175</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>18.76718807043834</v>
+        <v>18.76718799973135</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.338729368901232</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.971615790969407</v>
+        <v>1.971615791158568</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>66.48041229773915</v>
+        <v>66.48041227933734</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>18.78846758642689</v>
+        <v>18.78846760061245</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>3.149173955296404</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>1.080326531798915</v>
+        <v>1.080326531843429</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>59.91629660292053</v>
+        <v>59.91629662153535</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>40.68170850724233</v>
+        <v>40.68170836496233</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.4819305978692461</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>-0.6139914814953231</v>
+        <v>-0.6139914811330041</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>60.29870054369046</v>
+        <v>60.29870059519716</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>24.98394644805045</v>
+        <v>24.98394654847604</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>2.362406059829026</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.250040336967168</v>
+        <v>0.2500403369004036</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>622.1434527056908</v>
+        <v>622.1434527056909</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>176</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>48.08966605636832</v>
+        <v>48.08966603641047</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>10.45839242274422</v>
+        <v>10.45839239602317</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.8142018610892848</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>2.133042001704514</v>
+        <v>2.133042001927078</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>53.94947898935146</v>
+        <v>53.94947897840603</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>13.55749930884872</v>
+        <v>13.55749933895939</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.9492122845521752</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>15.2048653870319</v>
+        <v>15.20486538792179</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>45.45331487266832</v>
+        <v>45.45331496111965</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>20.63506351987064</v>
+        <v>20.63506362837203</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.2756028258529526</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.6882024399416053</v>
+        <v>0.6882024414672072</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>54.56344158402709</v>
+        <v>54.56344157956168</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>10.99413261058669</v>
+        <v>10.9941326213674</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.518855424708676</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>51.05015064328549</v>
+        <v>51.05015067064709</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>14.8468292270806</v>
+        <v>14.84682923297906</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.4210493135108956</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.305813846990998</v>
+        <v>0.3058138470688832</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>544.2830996629862</v>
+        <v>544.2830996629872</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>52</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>60.37878687716567</v>
+        <v>60.3787868208272</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>31.99474186974892</v>
+        <v>31.99474191263566</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.9532313968758288</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.0520269841545852</v>
+        <v>-0.052026984232482</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>59.69135439403221</v>
+        <v>59.69135438990824</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>19.73395333670786</v>
+        <v>19.73395333020756</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.7666533237050666</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.8572520668457677</v>
+        <v>0.8572520668568948</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>529.6376944217168</v>
+        <v>529.6376944217163</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>19.25</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>59.44043087441133</v>
+        <v>59.44043065761039</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>22.34597006240138</v>
+        <v>22.3459700738763</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.5206724268611933</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.2270408488769301</v>
+        <v>0.2270408489881987</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>50.91582480568743</v>
+        <v>50.91582474877895</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>18.10460676826045</v>
+        <v>18.10460679770882</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.7964605535242709</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.7698325272842919</v>
+        <v>0.7698325277293718</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>517.1719845022466</v>
+        <v>517.1719845022467</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>177.5</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>38.48379675166533</v>
+        <v>38.48379644629563</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26.49663408540461</v>
+        <v>26.49663422514935</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.5560296467548363</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.2317393876792808</v>
+        <v>0.2317393893483332</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>49.13971229947617</v>
+        <v>49.13971228828132</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>12.38334522544788</v>
+        <v>12.38334523823024</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.5217884528449944</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>1.55599321116014</v>
+        <v>1.555993211493959</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2170,21 +2170,21 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>8472</v>
+        <v>8086</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>夠麻吉</t>
+          <t>宏捷科</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>507.6981450770659</v>
+        <v>506.2219034568395</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>77</v>
+        <v>110.5</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>55.89240615643908</v>
+        <v>46.85430284762335</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.90917240461783</v>
+        <v>17.43990614002332</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.1014843986670705</v>
+        <v>0.4868624888069669</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.1018349689189352</v>
+        <v>0.4526778709392087</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>8086</v>
+        <v>8383</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>宏捷科</t>
+          <t>千附</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>506.2219034568387</v>
+        <v>504.3212564163193</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>110.5</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,16 +2248,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>46.85430270615146</v>
+        <v>52.55482960313283</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>17.43990615206165</v>
+        <v>10.84778784808645</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.4868624888069669</v>
+        <v>0.903921945478976</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.4526778719183997</v>
+        <v>0.4393550312982828</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>8383</v>
+        <v>8431</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>千附</t>
+          <t>匯鑽科</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>504.3212564163193</v>
+        <v>503.3234373475131</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>67.90000000000001</v>
+        <v>63.3</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>52.55482960313283</v>
+        <v>58.35674114672575</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>10.84778783566414</v>
+        <v>31.92187687598692</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.903921945478976</v>
+        <v>0.2089355531113578</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.4393550312204001</v>
+        <v>-0.2017804228860287</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>8431</v>
+        <v>8171</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>匯鑽科</t>
+          <t>天宇</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>503.323437347513</v>
+        <v>500.9975704306269</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>63.3</v>
+        <v>20.45</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,16 +2354,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>58.35674115005514</v>
+        <v>57.62345465743503</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>31.9218768695878</v>
+        <v>18.29721115164431</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.2089355531113578</v>
+        <v>0.6338296315688829</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.2017804227858861</v>
+        <v>0.0952041036053846</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>8171</v>
+        <v>8104</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>天宇</t>
+          <t>錸寶</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>500.9975704306268</v>
+        <v>488.2124552663787</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>20.45</v>
+        <v>31.05</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>57.6234546912795</v>
+        <v>52.21459610210344</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>18.29721115164431</v>
+        <v>18.59694273393671</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.6338296315688829</v>
+        <v>0.6853668817061258</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.0952041036387674</v>
+        <v>0.2262071887872546</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>8104</v>
+        <v>8466</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>錸寶</t>
+          <t>美吉吉-KY</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>488.2124552663785</v>
+        <v>487.3938393733867</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>31.05</v>
+        <v>15.6</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,16 +2460,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>52.2145962451758</v>
+        <v>54.59075884107726</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>18.59694262550056</v>
+        <v>39.45608901008254</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.6853668817061258</v>
+        <v>1.039383937338668</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.2262071884756947</v>
+        <v>0.2401357161719097</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>8466</v>
+        <v>8289</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>美吉吉-KY</t>
+          <t>泰藝</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>487.3938393733867</v>
+        <v>485.3203639330019</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>15.6</v>
+        <v>44.75</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>54.59075887482246</v>
+        <v>51.0126032432752</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>39.45608897673502</v>
+        <v>19.71298533132569</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1.039383937338668</v>
+        <v>1.422985645245699</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.2401357160940213</v>
+        <v>0.3214393282758121</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>8289</v>
+        <v>8131</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>泰藝</t>
+          <t>福懋科</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>485.3203639330019</v>
+        <v>472.4936819570752</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>44.75</v>
+        <v>61.4</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>51.01260325679139</v>
+        <v>48.78718444569376</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>19.71298532550243</v>
+        <v>8.687098737587711</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1.422985645245699</v>
+        <v>0.3914434129267762</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.3214393282090426</v>
+        <v>0.2640495954978767</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>8131</v>
+        <v>8097</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>福懋科</t>
+          <t>常珵</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>472.4936819570752</v>
+        <v>454.9226573483955</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>61.4</v>
+        <v>48.15</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>48.78718445367038</v>
+        <v>35.81790083235899</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>8.687098737587711</v>
+        <v>29.13454021476933</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.3914434129267762</v>
+        <v>0.3141820252078131</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.2640495954867552</v>
+        <v>0.1478936146172773</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>8097</v>
+        <v>8147</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>常珵</t>
+          <t>正淩</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>454.9226573483955</v>
+        <v>450.4610665738933</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>48.15</v>
+        <v>136.5</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>35.81790100832761</v>
+        <v>58.008292617515</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>29.13454026646765</v>
+        <v>21.86469610085332</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.3141820252078131</v>
+        <v>0.3750016215985811</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.147893614684037</v>
+        <v>0.53009083953767</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>8147</v>
+        <v>8472</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>正淩</t>
+          <t>夠麻吉</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>450.4610665738932</v>
+        <v>447.6981450770659</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>136.5</v>
+        <v>77</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>58.00829269030418</v>
+        <v>55.89240618114157</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>21.86469606300656</v>
+        <v>31.90917260832542</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.3750016215985811</v>
+        <v>0.1014843986670705</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.5300908392038342</v>
+        <v>0.1018349703877032</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>48.44972142045864</v>
+        <v>48.44972132119378</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>10.95986967101885</v>
+        <v>10.95986975437986</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.4941303244122554</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.168158395458887</v>
+        <v>0.168158395659175</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>27.60057458792417</v>
+        <v>27.6005745528172</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>36.30883208186607</v>
+        <v>36.30883208043576</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.7889698979822034</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.1463440612824502</v>
+        <v>-0.1463440611823063</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>444.1283470648083</v>
+        <v>444.128347064808</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>15.75</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>84.50422022572762</v>
+        <v>84.50422020029887</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>29.10211669148835</v>
+        <v>29.10211677453916</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.308481538430994</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.9629964311069878</v>
+        <v>0.9629964311260596</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>436.8096555749292</v>
+        <v>436.8096555749293</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>146</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>38.14435758542266</v>
+        <v>38.14435737114183</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>31.91448136341427</v>
+        <v>31.91448153847934</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.9161167786870856</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.9343161888691612</v>
+        <v>0.9343161903156734</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>17.52989328974989</v>
+        <v>17.52989294870693</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>25.9712066593548</v>
+        <v>25.97120687953185</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.523174251089526</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.9279283909892728</v>
+        <v>-0.9279283900768504</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>45.8344762770757</v>
+        <v>45.83447627357173</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>10.05367948770428</v>
+        <v>10.05367947871087</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.3889335063921308</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.1697988818661531</v>
+        <v>-0.1697988818216624</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>49.39066389075447</v>
+        <v>49.39066398761783</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>14.56543519005132</v>
+        <v>14.56543519485413</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.8553417803000599</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>42.37797740029435</v>
+        <v>42.37797733118728</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>14.29882069657826</v>
+        <v>14.29882061039096</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.5547481738671958</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.023374773851028</v>
+        <v>0.0233747739289165</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>39.11594069553625</v>
+        <v>39.1159406220659</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.01385831283155</v>
+        <v>22.01385828716402</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.4660050178545917</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.3324459166800244</v>
+        <v>-0.3324459164241058</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>425.0649577252809</v>
+        <v>425.064957725281</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>33.1</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>54.00722430554455</v>
+        <v>54.00722441157617</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>13.42631286137498</v>
+        <v>13.42631286343372</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5849108453482424</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0457724161142892</v>
+        <v>0.0457724160586522</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>44.21169467285982</v>
+        <v>44.21169462376707</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>15.6678378177548</v>
+        <v>15.66783785684134</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.009134458529496</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.09213944991292621</v>
+        <v>0.09213945001307321</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>49.37841332368541</v>
+        <v>49.37841340758519</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>30.95612488651591</v>
+        <v>30.95612490735817</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.056874129848251</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>51.51271464809114</v>
+        <v>51.51271464106846</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>15.87323203621415</v>
+        <v>15.87323199944272</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.6350891145931218</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.5955318745143826</v>
+        <v>0.5955318745811393</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.32676966813008</v>
+        <v>46.32676975755344</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>34.87387267196713</v>
+        <v>34.87387262242672</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>3.23385898973558</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.0267059016092799</v>
+        <v>-0.0267059016204078</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>26.65100557289973</v>
+        <v>26.65100542297285</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>39.7298797801257</v>
+        <v>39.7298798100277</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>3.649309215180266</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.1075793432542724</v>
+        <v>-0.1075793431541298</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>44.90268845807435</v>
+        <v>44.90268848966928</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>19.14537597398637</v>
+        <v>19.14537599682686</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.870816255095116</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.06862061057398899</v>
+        <v>0.0686206105480294</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>395.8062337398636</v>
+        <v>395.8062337398639</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>53.3</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>53.54616935921616</v>
+        <v>53.54616990012698</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>20.46370675379365</v>
+        <v>20.46370673505072</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.3461832113339587</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.5780893472119788</v>
+        <v>0.5780893465443543</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>44.80763023937629</v>
+        <v>44.80763040548378</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>22.13862430440547</v>
+        <v>22.13862430440548</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.1275646995738436</v>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>385.7957275390566</v>
+        <v>385.7957275390563</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>84.59999999999999</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>52.29123187603965</v>
+        <v>52.2912317687904</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>13.92391950789764</v>
+        <v>13.92391959303921</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.4376415564543019</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.5797672178506749</v>
+        <v>0.5797672180732227</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3788,7 +3788,7 @@
         <v>37.87423674067127</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>26.00549275485535</v>
+        <v>26.00549282108775</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.7153699446212035</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.7004082722255309</v>
+        <v>-0.7004082721142386</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,7 +3838,7 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>29.44608675179266</v>
+        <v>29.44608670018394</v>
       </c>
       <c r="I64" s="2" t="n">
         <v>17.94064223196193</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.07979653428492681</v>
+        <v>-0.0797965342737984</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>44.39218755379932</v>
+        <v>44.39218726052343</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>24.47278566422833</v>
+        <v>24.47278598163693</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.3123713669135161</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.1180622097301943</v>
+        <v>0.1180622100127113</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>365.5205522850393</v>
+        <v>365.5205522850394</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>372.5</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>50.21235909664376</v>
+        <v>50.21235901966063</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>14.87762766498431</v>
+        <v>14.87762768566612</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.4737584346274077</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0178239395518524</v>
+        <v>0.0178239404420496</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>362.918382004378</v>
+        <v>362.9183820043779</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>200</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>37.5937428339412</v>
+        <v>37.59374280275812</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>14.08524622068115</v>
+        <v>14.08524622531677</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.5345566382649994</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-1.382037487489757</v>
+        <v>-1.382037487333976</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.99986768959384</v>
+        <v>42.99986756018126</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>50.12267887742955</v>
+        <v>50.12267895307647</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.1325957316254722</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.0095658035633331</v>
+        <v>0.0095658035522075</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>45.4685263260832</v>
+        <v>45.46852632392009</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>19.50820935580382</v>
+        <v>19.50820932452053</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.280201857278177</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-6.479680302953822</v>
+        <v>-6.479680302987227</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4159,7 +4159,7 @@
         <v>63.31744515112216</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>24.26062797343563</v>
+        <v>24.26062856539176</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.8319893985992698</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.602396771924833</v>
+        <v>0.602396772363443</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>39.94508779821312</v>
+        <v>39.9450875491713</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>10.85102128183244</v>
+        <v>10.85102142341535</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>1.639268796293905</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.1751220949256044</v>
+        <v>-0.1751220946140431</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>330.0126788458994</v>
+        <v>330.0126788458995</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>35.15</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>39.99564296981912</v>
+        <v>39.99564306593176</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>12.69420564312602</v>
+        <v>12.69420570357059</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.2304158707798676</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0136642316974699</v>
+        <v>0.0136642317642322</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>328.9823309030292</v>
+        <v>328.9823309030287</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>8.43</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>48.51368793679789</v>
+        <v>48.51368782548809</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.41996240304545</v>
+        <v>14.41996238712349</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5661568193279873</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.0251797276297151</v>
+        <v>-0.0251797276052353</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>324.0653797337834</v>
+        <v>324.0653797337835</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>47.05</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>48.07242049017137</v>
+        <v>48.07242038295151</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>4.145683057586741</v>
+        <v>4.14568299208878</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.2683088038008233</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.1784949681699747</v>
+        <v>-0.1784949677026407</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>49.23799436999335</v>
+        <v>49.237994397423</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>14.05429551752357</v>
+        <v>14.05429551392951</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.445763561849045</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.1408165623425273</v>
+        <v>-0.1408165625141591</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>53.52631451143581</v>
+        <v>53.52631453450378</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>23.99762039925318</v>
+        <v>23.99762040722103</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.4103483784851667</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.0079777637337949</v>
+        <v>-0.007977763722666099</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>37.81261868001484</v>
+        <v>37.81261882540478</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>21.42950274884439</v>
+        <v>21.42950280333696</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.4644478450351711</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.358876862792586</v>
+        <v>-0.3588768633489492</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>39.93312466672375</v>
+        <v>39.93312488911993</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>10.24727622473863</v>
+        <v>10.24727642059358</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.7516525806234273</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.0658733109083447</v>
+        <v>-0.0658733107176481</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>296.3144639469753</v>
+        <v>296.3144639469752</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>23.25</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>49.16335520934196</v>
+        <v>49.16335521372047</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7.24664055793403</v>
+        <v>7.246640572970472</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>3.345345107511979</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.3995026818081206</v>
+        <v>0.3995026817747367</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.15242467027045</v>
+        <v>42.15242449344301</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>24.42146607147134</v>
+        <v>24.42146612886344</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.9397689835009752</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0410481150486006</v>
+        <v>0.04104811512649</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>294.7810684346021</v>
+        <v>294.7810684346022</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>254.5</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>51.21914761923617</v>
+        <v>51.21914760956194</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>10.43097166609611</v>
+        <v>10.43097172565194</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.3878861441404991</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>3.728766872936596</v>
+        <v>3.728766872046448</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>48.32425290956479</v>
+        <v>48.32425284212484</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>21.58218233772048</v>
+        <v>21.58218232597822</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.681370007962677</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.0222265795079443</v>
+        <v>-0.022226579530198</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>293.4227255962333</v>
+        <v>293.4227255962334</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>20.25</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>54.23503458490082</v>
+        <v>54.23503412320312</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>12.44793143758672</v>
+        <v>12.44793145813562</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.6877823844440697</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0352277485601328</v>
+        <v>0.0352277486491523</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>42.55863151753066</v>
+        <v>42.55863146802231</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>42.72641316036842</v>
+        <v>42.72641324019654</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.3932362014188735</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.1363682499579219</v>
+        <v>-0.1363682499690494</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.36201773216294</v>
+        <v>47.36201784967732</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>15.23019304094662</v>
+        <v>15.23019310985022</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.5436892434893971</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.2053828622081999</v>
+        <v>0.2053828619967879</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>286.8794301485563</v>
+        <v>286.8794301485561</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>39.4</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>39.19199908639152</v>
+        <v>39.19199913717388</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>30.92056735080586</v>
+        <v>30.92056736449721</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4600448014237869</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.0868122731771603</v>
+        <v>-0.0868122732327942</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>283.2902910665772</v>
+        <v>283.2902910665771</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>897</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>39.97071587968107</v>
+        <v>39.97071584927116</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>18.6583454423136</v>
+        <v>18.65834544635107</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.444930927993597</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>4.895038579615424</v>
+        <v>4.895038582953703</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.40131516414796</v>
+        <v>50.40131479909326</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>9.462408584554872</v>
+        <v>9.462408589937974</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.362856786976976</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.292590356136892</v>
+        <v>0.2925903562481678</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>44.96081753811517</v>
+        <v>44.96081995665166</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>7.444581354142318</v>
+        <v>7.44458223692283</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.325644556652131</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.1218043634720291</v>
+        <v>-0.1218043665876256</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>37.20028003686538</v>
+        <v>37.20028002788251</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>17.52253043556248</v>
+        <v>17.52253044032677</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3903558381112108</v>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>263.5209055461641</v>
+        <v>263.5209055461643</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>9.19</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>28.350882717278</v>
+        <v>28.35088269732634</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>19.03659352802887</v>
+        <v>19.03659347461897</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.7000221883848787</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.0540444505472132</v>
+        <v>-0.0540444505427621</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>260.8136734565914</v>
+        <v>260.8136734565915</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>4.97</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.44134766064969</v>
+        <v>41.44134762219031</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>11.72281974578208</v>
+        <v>11.72281978144088</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.5838453257311198</v>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>258.5109764670899</v>
+        <v>258.51097646709</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>32.6</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>54.62830472869088</v>
+        <v>54.62830490540274</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>21.711223276586</v>
+        <v>21.71122339830848</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.5051521165819309</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.2944629124362764</v>
+        <v>0.2944629125364201</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>42.15212434322965</v>
+        <v>42.15212417856723</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>10.22696184385858</v>
+        <v>10.22696190573423</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.6874965859140107</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.6320824964760692</v>
+        <v>0.6320824970324121</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>248.6730044516942</v>
+        <v>248.6730044516941</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>19.5</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.77982143445032</v>
+        <v>44.77982140952909</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>8.390137098795051</v>
+        <v>8.39013706659626</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.245561382279997</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0439821997500337</v>
+        <v>0.0439821997277802</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>246.6614371408465</v>
+        <v>246.6614371408461</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>12.9</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>49.19606336536266</v>
+        <v>49.19606362317047</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>14.77667112214393</v>
+        <v>14.7766710425782</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.7997761087847904</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0314301622346051</v>
+        <v>0.0314301619564271</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>236.4057042949894</v>
+        <v>236.4057042949891</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>75.3</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>37.77160691931539</v>
+        <v>37.77160675302839</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>9.398379834089996</v>
+        <v>9.398379831011146</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.5825787599634195</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.3036527534780893</v>
+        <v>-0.3036527531442794</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>42.39432402529686</v>
+        <v>42.39432405021238</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.44583043540398</v>
+        <v>19.44583044367304</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.2746056498663073</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.060624620080856</v>
+        <v>0.0606246200697297</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>49.27768869904094</v>
+        <v>49.27768900031964</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>11.10051421895303</v>
+        <v>11.10051427958877</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4367841844436976</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.0177174192611581</v>
+        <v>-0.0177174193613043</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>221.7109784126366</v>
+        <v>221.7109784126372</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>60.4</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>28.49669415520654</v>
+        <v>28.49669396199074</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>24.98660349158245</v>
+        <v>24.98660369663632</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>1.114162322787678</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.1237534030931438</v>
+        <v>-0.1237534029596162</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>215.5981214848344</v>
+        <v>215.5981214848345</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>89</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>44.68622278483763</v>
+        <v>44.68622268780207</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>9.332393963251448</v>
+        <v>9.332394101580748</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.2162697450883984</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.7027044996083918</v>
+        <v>0.7027045009436423</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>212.1969358151012</v>
+        <v>212.1969358151014</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>13.55</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>24.54647942493584</v>
+        <v>24.5464794395908</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>41.99963469366903</v>
+        <v>41.99963466240234</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.5310955820293388</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0760036264172663</v>
+        <v>-0.0760036264617731</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>202.549062215144</v>
+        <v>202.5490622151442</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>5.89</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>38.14936230372392</v>
+        <v>38.14936252377669</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>6.846930116590902</v>
+        <v>6.846930084278321</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.7314112182093602</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.002918032386262</v>
+        <v>-0.002918032395164</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>198.0694103217371</v>
+        <v>198.0694103217369</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>39.35</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>46.09363210247465</v>
+        <v>46.09363209106856</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>19.94950435419418</v>
+        <v>19.94950437178924</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.3511471031230672</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.2198410525403364</v>
+        <v>0.2198410526070982</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>194.5652561574584</v>
+        <v>194.5652561574585</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>59.5</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>49.54884807764718</v>
+        <v>49.54884799905644</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>5.337048992811719</v>
+        <v>5.33704970677725</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.323697974993742</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.6725043825877528</v>
+        <v>0.6725043845683829</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>51.62588035612842</v>
+        <v>51.62588065507413</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>5.658894241647873</v>
+        <v>5.658894228318797</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.502593681593569</v>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>172.0823473596238</v>
+        <v>172.0823473596233</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>40.6</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>49.6493864620535</v>
+        <v>49.64938630871612</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>19.08263474226872</v>
+        <v>19.08263475670941</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.5495948264807</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0385472033091658</v>
+        <v>-0.0385472032757795</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>161.3857762199506</v>
+        <v>161.3857762199497</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>23</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>36.18675101559953</v>
+        <v>36.18675094586742</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>8.986110963551734</v>
+        <v>8.986110896786725</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.893659418827158</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.0297630655547189</v>
+        <v>-0.0297630655213343</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>157.1080846606431</v>
+        <v>157.1080846606432</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>90</v>
@@ -6226,7 +6226,7 @@
         <v>33.45243353613918</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>18.48180991696254</v>
+        <v>18.48180998492158</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.896578083115382</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.3328505606053737</v>
+        <v>-0.3328505605831247</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>149.8091051196774</v>
+        <v>149.8091051196775</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>51</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>43.72465858264421</v>
+        <v>43.72465859494889</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>18.5209253213688</v>
+        <v>18.52092525443952</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.5276458726983252</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.1175650213485337</v>
+        <v>0.1175650213374135</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>38.27480375700789</v>
+        <v>38.27480378456713</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>12.6822608357452</v>
+        <v>12.68226081517785</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.5723249928578833</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.1690291715078911</v>
+        <v>0.1690291715635312</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.99380961031101</v>
+        <v>44.99380938776757</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>15.63720279968348</v>
+        <v>15.63720291759082</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.2395428548505835</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1369212736060691</v>
+        <v>0.1369212737507225</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>45.39913048590408</v>
+        <v>45.39913045343331</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>18.10598995760498</v>
+        <v>18.10598996055602</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.8672114889065011</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.0318615844428749</v>
+        <v>-0.0318615843316032</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>41.91379303473207</v>
+        <v>41.91379296991716</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>14.48992259528953</v>
+        <v>14.48992263530714</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6894388878350682</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0357975575094761</v>
+        <v>0.0357975575762384</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>110.6111934021031</v>
+        <v>110.6111934021034</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>15</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>47.42784351015117</v>
+        <v>47.42784314278963</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>9.467741822170172</v>
+        <v>9.467741862556064</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.3103001592981505</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.0435106232384894</v>
+        <v>0.0435106233608864</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>89.01903852085742</v>
+        <v>89.01903852085738</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>139.5</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.64614018545959</v>
+        <v>39.64613988448409</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>8.293373572828507</v>
+        <v>8.293373642979414</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.8931317648877506</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0143216914529054</v>
+        <v>0.0143216911191208</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>51.17171169739495</v>
+        <v>51.17171185907385</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>17.29657476797866</v>
+        <v>17.29657484085701</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.3036550859683092</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1788009435729169</v>
+        <v>-0.1788009436062991</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>

</xml_diff>